<commit_message>
ajout de depanage en dev web/js
</commit_message>
<xml_diff>
--- a/feuille-de-calcul.xlsx
+++ b/feuille-de-calcul.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="75">
   <si>
     <t>Commentaires</t>
   </si>
@@ -324,6 +324,51 @@
   </si>
   <si>
     <t>Developpement web javascript</t>
+  </si>
+  <si>
+    <t>Refus de push (repository different)</t>
+  </si>
+  <si>
+    <t>rejected (fetch first)</t>
+  </si>
+  <si>
+    <t>Le depot distant contenait déjà des fichiers differents du local</t>
+  </si>
+  <si>
+    <t>Cas typique quand on initialise Github avant le local</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> exemple 6</t>
+  </si>
+  <si>
+    <t>Conflit de fusion sur un fichier</t>
+  </si>
+  <si>
+    <t>Le meme fichier (tailwindcss/output,css) a été cree separement en local et sur Github</t>
+  </si>
+  <si>
+    <t>Resoudre le conflit (editer ou choisir version) puis git add,git commit</t>
+  </si>
+  <si>
+    <t>git pull origin main --allow-unrelated-histories</t>
+  </si>
+  <si>
+    <t>Github + Git</t>
+  </si>
+  <si>
+    <t>Dgit/Conflit</t>
+  </si>
+  <si>
+    <t>CONFLIT (add/add)</t>
+  </si>
+  <si>
+    <t>Editeur de code (VS Code)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichier generer ,a ignorer normalement </t>
+  </si>
+  <si>
+    <t>exemple 7_</t>
   </si>
 </sst>
 </file>
@@ -1200,11 +1245,54 @@
       <c r="B7" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="F7" s="4"/>
-    </row>
-    <row r="8" spans="1:9" ht="22.8">
+      <c r="C7" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="40.799999999999997">
       <c r="A8" s="5"/>
-      <c r="F8" s="4"/>
+      <c r="B8" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="9" spans="1:9" ht="22.8">
       <c r="A9" s="5"/>
@@ -1828,6 +1916,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -2050,36 +2153,10 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2102,9 +2179,20 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
ajout du depannage de aws lambda sur l'echec d'execution d'extraction de la base de donnees Mysql
</commit_message>
<xml_diff>
--- a/feuille-de-calcul.xlsx
+++ b/feuille-de-calcul.xlsx
@@ -356,9 +356,6 @@
     <t>Github + Git</t>
   </si>
   <si>
-    <t>Dgit/Conflit</t>
-  </si>
-  <si>
     <t>CONFLIT (add/add)</t>
   </si>
   <si>
@@ -369,6 +366,9 @@
   </si>
   <si>
     <t>exemple 7_</t>
+  </si>
+  <si>
+    <t>git/Conflit</t>
   </si>
 </sst>
 </file>
@@ -1269,14 +1269,14 @@
     </row>
     <row r="8" spans="1:9" ht="40.799999999999997">
       <c r="A8" s="5"/>
-      <c r="B8" s="4" t="s">
-        <v>70</v>
+      <c r="B8" s="25" t="s">
+        <v>74</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>65</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E8" s="4" t="s">
         <v>66</v>
@@ -1285,13 +1285,13 @@
         <v>67</v>
       </c>
       <c r="G8" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>72</v>
       </c>
-      <c r="H8" s="4" t="s">
+      <c r="I8" s="3" t="s">
         <v>73</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="22.8">

</xml_diff>

<commit_message>
changement de version de mariadb dans le lab de migration de amazon RDS
</commit_message>
<xml_diff>
--- a/feuille-de-calcul.xlsx
+++ b/feuille-de-calcul.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="94">
   <si>
     <t>Commentaires</t>
   </si>
@@ -365,17 +365,74 @@
     <t xml:space="preserve">Fichier generer ,a ignorer normalement </t>
   </si>
   <si>
-    <t>exemple 7_</t>
-  </si>
-  <si>
     <t>git/Conflit</t>
+  </si>
+  <si>
+    <t>exemple 7</t>
+  </si>
+  <si>
+    <t>Ex-7</t>
+  </si>
+  <si>
+    <t>Ex-8</t>
+  </si>
+  <si>
+    <t>AWS Lambda</t>
+  </si>
+  <si>
+    <t>Echec de l'execution sur l'extraction des donnees dans la base de donnees</t>
+  </si>
+  <si>
+    <t>Un message d'erreur s'affiche</t>
+  </si>
+  <si>
+    <t>Les regles entrantes du groupe de securite utilisees par l'instance EC2 ne contiennent pas le numero de port de MySql</t>
+  </si>
+  <si>
+    <t>Entrer dans VPC,cliquer sur le lien du groupe de securite et modifier les regles entrantes  en ajouter le port 3306 de MySql/Aurora</t>
+  </si>
+  <si>
+    <t>VPC,groupe de securite</t>
+  </si>
+  <si>
+    <t>echec d'execution lorsqu'on met pas les regles entrants</t>
+  </si>
+  <si>
+    <t>exemple-8</t>
+  </si>
+  <si>
+    <t>Ex-9</t>
+  </si>
+  <si>
+    <t>Migrer vers Amazon RDS</t>
+  </si>
+  <si>
+    <t>Echec de la creation de l'instance de Amazon RDS pour MariaDB</t>
+  </si>
+  <si>
+    <t>Apres l'execution de la commande de creation de l'instance,un message d'erreur s'affiche(invalidation de la combinaison des parametres)</t>
+  </si>
+  <si>
+    <t>"Une erreur s’est produite (combinaison de paramètres invalide) lors de l’appel de l’opération CreateDBInstance : impossible de trouver la version 10.5.13 pour MariaDB."</t>
+  </si>
+  <si>
+    <t>Nous avons changer la version de mariaDb,passant de 10.15.13 a 10.15.27</t>
+  </si>
+  <si>
+    <t>Se connecter a l'instance cafeInstance</t>
+  </si>
+  <si>
+    <t>La version qui nous a été proposer dans le lab n'est pas la bonne</t>
+  </si>
+  <si>
+    <t>exemple-9</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="16">
+  <fonts count="18">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -475,6 +532,18 @@
       <b/>
       <sz val="18"/>
       <color theme="0"/>
+      <name val="Amazon Ember"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="9"/>
+      <name val="Amazon Ember"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FFFF0000"/>
       <name val="Amazon Ember"/>
     </font>
   </fonts>
@@ -631,7 +700,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -712,6 +781,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1242,7 +1317,7 @@
       <c r="A7" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="25" t="s">
+      <c r="B7" s="28" t="s">
         <v>58</v>
       </c>
       <c r="C7" s="4" t="s">
@@ -1268,9 +1343,11 @@
       </c>
     </row>
     <row r="8" spans="1:9" ht="40.799999999999997">
-      <c r="A8" s="5"/>
-      <c r="B8" s="25" t="s">
-        <v>74</v>
+      <c r="A8" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="28" t="s">
+        <v>73</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>65</v>
@@ -1291,15 +1368,66 @@
         <v>72</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="22.8">
-      <c r="A9" s="5"/>
-      <c r="F9" s="4"/>
-    </row>
-    <row r="10" spans="1:9" ht="22.8">
-      <c r="A10" s="5"/>
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="81.599999999999994">
+      <c r="A9" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="B9" s="29" t="s">
+        <v>77</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="81.599999999999994">
+      <c r="A10" s="5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B10" s="29" t="s">
+        <v>86</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="I10" s="3" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="11" spans="1:9" ht="22.8">
       <c r="A11" s="5"/>

</xml_diff>

<commit_message>
ajout des confilts rencontrer sur devops
</commit_message>
<xml_diff>
--- a/feuille-de-calcul.xlsx
+++ b/feuille-de-calcul.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="110">
   <si>
     <t>Commentaires</t>
   </si>
@@ -287,9 +287,6 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve"> </t>
-  </si>
-  <si>
     <t>Ex-5</t>
   </si>
   <si>
@@ -426,13 +423,88 @@
   </si>
   <si>
     <t>exemple-9</t>
+  </si>
+  <si>
+    <t>Ex-10</t>
+  </si>
+  <si>
+    <t>DevOps</t>
+  </si>
+  <si>
+    <t>Error: ENOENT: no such file or directory, stat '/app/Frontend/public/index.html'</t>
+  </si>
+  <si>
+    <t>Le Backend original (app.js) essayait de servir les fichiers Frontend, mais dans Docker ils sont dans des conteneurs séparés</t>
+  </si>
+  <si>
+    <t>Le backend ne parvenait pas a communiquer avec le frontend</t>
+  </si>
+  <si>
+    <t>cree app.docker.js une version speciale de Docker (API seulement),Modifier Backend/Dokerfile pour utiliser app.docker.js au lieu de app.js</t>
+  </si>
+  <si>
+    <t>Docker</t>
+  </si>
+  <si>
+    <t>Ex-11</t>
+  </si>
+  <si>
+    <t>Backend lance Ngnix au lieu de Node.js</t>
+  </si>
+  <si>
+    <t>les logs montraient:portfolio-backend | nginx/1.29.8
+portfolio-backend | start worker processes</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Docker utilisait l'ancien cache/image qui contenait encore l'ancienne configuration</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Forcer la reconstruction sans cache: </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Amazon Ember"/>
+      </rPr>
+      <t>docker-compose down
+docker-compose build --no-cache backend
+docker-compose up -d</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="16"/>
+        <color theme="1"/>
+        <rFont val="Amazon Ember"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+  </si>
+  <si>
+    <t>API,node,configuration,docker</t>
+  </si>
+  <si>
+    <t>exemple 10</t>
+  </si>
+  <si>
+    <t>exemple 11</t>
+  </si>
+  <si>
+    <t>Situation : Application originale = 1 serveur Node.js servant API + fichiers statiques                                                      Problème Docker : Chaque conteneur est isolé → Backend ne trouve plus les fichiers Frontend</t>
+  </si>
+  <si>
+    <t>Logs Nginx au lieu de Node.js → Cache Docker utilisait ancienne image</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="18">
+  <fonts count="19">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -544,6 +616,12 @@
       <b/>
       <sz val="16"/>
       <color rgb="FFFF0000"/>
+      <name val="Amazon Ember"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="20"/>
+      <color theme="4"/>
       <name val="Amazon Ember"/>
     </font>
   </fonts>
@@ -700,7 +778,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -788,6 +866,12 @@
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -1286,160 +1370,210 @@
     </row>
     <row r="6" spans="1:9" ht="81.599999999999994">
       <c r="A6" s="26" t="s">
+        <v>47</v>
+      </c>
+      <c r="B6" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="25" t="s">
+      <c r="C6" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="27" t="s">
         <v>50</v>
       </c>
-      <c r="D6" s="27" t="s">
+      <c r="E6" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>52</v>
       </c>
-      <c r="F6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G6" s="4" t="s">
+      <c r="H6" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="H6" s="4" t="s">
+      <c r="I6" s="3" t="s">
         <v>55</v>
-      </c>
-      <c r="I6" s="3" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="7" spans="1:9" ht="42">
       <c r="A7" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="B7" s="28" t="s">
-        <v>58</v>
-      </c>
       <c r="C7" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="D7" s="3" t="s">
+      <c r="E7" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="F7" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="H7" s="4" t="s">
+      <c r="I7" s="3" t="s">
         <v>63</v>
-      </c>
-      <c r="I7" s="3" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="40.799999999999997">
       <c r="A8" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B8" s="28" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="I8" s="3" t="s">
         <v>73</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>65</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="I8" s="3" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="81.599999999999994">
       <c r="A9" s="5" t="s">
+        <v>75</v>
+      </c>
+      <c r="B9" s="29" t="s">
         <v>76</v>
       </c>
-      <c r="B9" s="29" t="s">
+      <c r="C9" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>78</v>
       </c>
-      <c r="D9" s="3" t="s">
+      <c r="E9" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="4" t="s">
         <v>80</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="G9" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="G9" s="3" t="s">
+      <c r="H9" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="I9" s="3" t="s">
         <v>83</v>
-      </c>
-      <c r="I9" s="3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="81.599999999999994">
       <c r="A10" s="5" t="s">
+        <v>84</v>
+      </c>
+      <c r="B10" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="B10" s="29" t="s">
+      <c r="C10" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="D10" s="4" t="s">
         <v>87</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>88</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="F10" s="4" t="s">
         <v>89</v>
       </c>
-      <c r="F10" s="4" t="s">
+      <c r="G10" s="4" t="s">
         <v>90</v>
       </c>
-      <c r="G10" s="4" t="s">
+      <c r="H10" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="H10" s="4" t="s">
+      <c r="I10" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="I10" s="3" t="s">
+    </row>
+    <row r="11" spans="1:9" ht="122.4">
+      <c r="A11" s="5" t="s">
         <v>93</v>
       </c>
-    </row>
-    <row r="11" spans="1:9" ht="22.8">
-      <c r="A11" s="5"/>
-      <c r="F11" s="3" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="22.8">
-      <c r="A12" s="5"/>
+      <c r="B11" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="F11" s="31" t="s">
+        <v>98</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="I11" s="3" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="105">
+      <c r="A12" s="5" t="s">
+        <v>100</v>
+      </c>
+      <c r="B12" s="30" t="s">
+        <v>94</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>103</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>109</v>
+      </c>
+      <c r="I12" s="3" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="22.8">
       <c r="A13" s="5"/>
+      <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:9" ht="22.8">
       <c r="A14" s="5"/>
@@ -2029,12 +2163,12 @@
     </row>
     <row r="10" spans="2:2">
       <c r="B10" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="11" spans="2:2">
       <c r="B11" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>
@@ -2044,21 +2178,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x01010006807B066C556C4DA1F97EE96CC1104B" ma:contentTypeVersion="13" ma:contentTypeDescription="Utwórz nowy dokument." ma:contentTypeScope="" ma:versionID="cfb987611df5cdae7f7a5067c3395bc7">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c2ee6f6c-285d-4b95-ace0-9682ebe56039" xmlns:ns3="012b183d-1ada-4ff6-b855-98c4d59bda2b" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="08f2586826dc5d0b05e832f2b79fc23a" ns2:_="" ns3:_="">
     <xsd:import namespace="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
@@ -2281,10 +2400,36 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
+    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -2307,20 +2452,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E55E6835-5439-4B85-9C34-8A416D678E4C}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C795275D-8D89-4504-820D-42600FA03DDE}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="c2ee6f6c-285d-4b95-ace0-9682ebe56039"/>
-    <ds:schemaRef ds:uri="012b183d-1ada-4ff6-b855-98c4d59bda2b"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>